<commit_message>
Use non-zero values in FoGBPD and correct CA 45X implementation
</commit_message>
<xml_diff>
--- a/InputData/elec/FoGBPD/Fraction of Grid Batteries Produced Domestically.xlsx
+++ b/InputData/elec/FoGBPD/Fraction of Grid Batteries Produced Domestically.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\FoGBPD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A13247-FEEE-452A-8071-57B0D0178465}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D9D623-6155-44F0-814D-980B3CD49663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{DC12087C-9A27-4A43-B4A9-6B3F1E517F08}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -137,7 +137,7 @@
     </xf>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -521,17 +521,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF982137-6F01-4109-8226-D4C6F3731BA9}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="101.26953125" customWidth="1"/>
+    <col min="2" max="2" width="101.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -539,40 +539,40 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B4" s="2">
         <v>2024</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -585,19 +585,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13AB29A9-70CB-4471-AE81-9A64EFDA202F}">
   <dimension ref="B21:B24"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="4">
         <v>0.62</v>
       </c>
@@ -613,231 +613,203 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AA2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.54296875" customWidth="1"/>
-    <col min="6" max="6" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.5703125" customWidth="1"/>
+    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1">
-        <v>2021</v>
+        <v>2025</v>
       </c>
       <c r="C1">
-        <v>2022</v>
+        <v>2026</v>
       </c>
       <c r="D1">
-        <v>2023</v>
+        <v>2027</v>
       </c>
       <c r="E1">
-        <v>2024</v>
+        <v>2028</v>
       </c>
       <c r="F1">
-        <v>2025</v>
+        <v>2029</v>
       </c>
       <c r="G1">
-        <v>2026</v>
+        <v>2030</v>
       </c>
       <c r="H1">
-        <v>2027</v>
+        <v>2031</v>
       </c>
       <c r="I1">
-        <v>2028</v>
+        <v>2032</v>
       </c>
       <c r="J1">
-        <v>2029</v>
+        <v>2033</v>
       </c>
       <c r="K1">
-        <v>2030</v>
+        <v>2034</v>
       </c>
       <c r="L1">
-        <v>2031</v>
+        <v>2035</v>
       </c>
       <c r="M1">
-        <v>2032</v>
+        <v>2036</v>
       </c>
       <c r="N1">
-        <v>2033</v>
+        <v>2037</v>
       </c>
       <c r="O1">
-        <v>2034</v>
+        <v>2038</v>
       </c>
       <c r="P1">
-        <v>2035</v>
+        <v>2039</v>
       </c>
       <c r="Q1">
-        <v>2036</v>
+        <v>2040</v>
       </c>
       <c r="R1">
-        <v>2037</v>
+        <v>2041</v>
       </c>
       <c r="S1">
-        <v>2038</v>
+        <v>2042</v>
       </c>
       <c r="T1">
-        <v>2039</v>
+        <v>2043</v>
       </c>
       <c r="U1">
-        <v>2040</v>
+        <v>2044</v>
       </c>
       <c r="V1">
-        <v>2041</v>
+        <v>2045</v>
       </c>
       <c r="W1">
-        <v>2042</v>
+        <v>2046</v>
       </c>
       <c r="X1">
-        <v>2043</v>
+        <v>2047</v>
       </c>
       <c r="Y1">
-        <v>2044</v>
+        <v>2048</v>
       </c>
       <c r="Z1">
-        <v>2045</v>
+        <v>2049</v>
       </c>
       <c r="AA1">
-        <v>2046</v>
-      </c>
-      <c r="AB1">
-        <v>2047</v>
-      </c>
-      <c r="AC1">
-        <v>2048</v>
-      </c>
-      <c r="AD1">
-        <v>2049</v>
-      </c>
-      <c r="AE1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" s="3" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="6">
-        <f>'S&amp;P'!B24</f>
+        <f>'S&amp;P'!$B$24</f>
         <v>0.62</v>
       </c>
       <c r="C2" s="6">
-        <f>'S&amp;P'!C24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="D2" s="6">
-        <f>'S&amp;P'!D24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="E2" s="6">
-        <f>'S&amp;P'!E24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="F2" s="6">
-        <f>'S&amp;P'!F24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="G2" s="6">
-        <f>'S&amp;P'!G24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="H2" s="6">
-        <f>'S&amp;P'!H24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="I2" s="6">
-        <f>'S&amp;P'!I24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="J2" s="6">
-        <f>'S&amp;P'!J24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="K2" s="6">
-        <f>'S&amp;P'!K24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="L2" s="6">
-        <f>'S&amp;P'!L24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="M2" s="6">
-        <f>'S&amp;P'!M24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="N2" s="6">
-        <f>'S&amp;P'!N24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="O2" s="6">
-        <f>'S&amp;P'!O24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="P2" s="6">
-        <f>'S&amp;P'!P24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="Q2" s="6">
-        <f>'S&amp;P'!Q24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="R2" s="6">
-        <f>'S&amp;P'!R24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="S2" s="6">
-        <f>'S&amp;P'!S24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="T2" s="6">
-        <f>'S&amp;P'!T24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="U2" s="6">
-        <f>'S&amp;P'!U24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="V2" s="6">
-        <f>'S&amp;P'!V24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="W2" s="6">
-        <f>'S&amp;P'!W24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="X2" s="6">
-        <f>'S&amp;P'!X24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="Y2" s="6">
-        <f>'S&amp;P'!Y24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="Z2" s="6">
-        <f>'S&amp;P'!Z24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
       <c r="AA2" s="6">
-        <f>'S&amp;P'!AA24</f>
-        <v>0</v>
-      </c>
-      <c r="AB2" s="6">
-        <f>'S&amp;P'!AB24</f>
-        <v>0</v>
-      </c>
-      <c r="AC2" s="6">
-        <f>'S&amp;P'!AC24</f>
-        <v>0</v>
-      </c>
-      <c r="AD2" s="6">
-        <f>'S&amp;P'!AD24</f>
-        <v>0</v>
-      </c>
-      <c r="AE2" s="6">
-        <f>'S&amp;P'!AE24</f>
-        <v>0</v>
+        <f>'S&amp;P'!$B$24</f>
+        <v>0.62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>